<commit_message>
Worked on CSS, fixed some different elements across pages
Our CSS is mostly done. We have met all of the basic requirements, but likely want to spend some more time making the site look better. My next step will be making sure all pages have the same header link (back to the home page) and doing other QA work before continuing to mess with the CSS.
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker (2).xlsx
+++ b/CSCI330 Group Project Task Tracker (2).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/904877C71E702AD1/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD93DA79-E5DC-4A71-85C3-BFCC4288317A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
   <si>
     <t>Task</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>need to apply css</t>
+  </si>
+  <si>
+    <t>Maisee, Beatrice</t>
   </si>
 </sst>
 </file>
@@ -498,16 +501,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4840B388-0DE6-4C53-AF10-25A76A976816}">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" customWidth="1"/>
-    <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -524,7 +527,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -542,7 +545,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -559,7 +562,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -569,8 +572,11 @@
       <c r="C4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D4" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -588,7 +594,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -596,10 +602,13 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -607,15 +616,18 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -625,7 +637,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -642,7 +654,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -653,7 +665,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -664,7 +676,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Updates for Module 2 Tracker
</commit_message>
<xml_diff>
--- a/CSCI330 Group Project Task Tracker (2).xlsx
+++ b/CSCI330 Group Project Task Tracker (2).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://marietta0-my.sharepoint.com/personal/mca003_marietta_edu/Documents/Junior Year/F26/CSCI330/Group Project/Web-Design-and-Programming-GroupWork/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD93DA79-E5DC-4A71-85C3-BFCC4288317A}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{DA7DD34A-3871-4552-B4C9-0B224A20E188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F6A5FAB-AFE7-47E1-ACB1-A9D1F95A9BF3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{35008FAE-AE0E-4657-A8AE-48045A98CB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="41">
   <si>
     <t>Task</t>
   </si>
@@ -117,13 +117,58 @@
   </si>
   <si>
     <t>Maisee, Beatrice</t>
+  </si>
+  <si>
+    <t>MODULE TWO</t>
+  </si>
+  <si>
+    <t>Enroll Student form display</t>
+  </si>
+  <si>
+    <t>Add Instructor form display</t>
+  </si>
+  <si>
+    <t>Add Course form display</t>
+  </si>
+  <si>
+    <t>Register Course form display</t>
+  </si>
+  <si>
+    <t>Drop Course form display</t>
+  </si>
+  <si>
+    <t>Updating manuals</t>
+  </si>
+  <si>
+    <t>Update select list display for Add Course</t>
+  </si>
+  <si>
+    <t>Enroll Student validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Instructor validation (4 rules)</t>
+  </si>
+  <si>
+    <t>Add Course validation (9 rules)</t>
+  </si>
+  <si>
+    <t>Register Course validation (6 rules)</t>
+  </si>
+  <si>
+    <t>Drop Course validation (6 rules)</t>
+  </si>
+  <si>
+    <t>Beatrice &amp; Maisee</t>
+  </si>
+  <si>
+    <t>Any updates/fixes from Module 1 grade</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,6 +184,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -148,7 +201,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -156,16 +209,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,10 +574,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4840B388-0DE6-4C53-AF10-25A76A976816}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" customWidth="1"/>
     <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
@@ -602,7 +676,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2">
         <v>46285</v>
@@ -616,7 +690,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D7" s="2">
         <v>46285</v>
@@ -630,7 +704,7 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2">
         <f>DATE(2026,9,17)</f>
@@ -662,7 +736,7 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -673,7 +747,7 @@
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -684,10 +758,198 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C12" xr:uid="{1AE900CF-695F-49FE-919B-A3667E9EEDD6}">
       <formula1>"Not started, In progress, Completed, Stuck/need help"</formula1>

</xml_diff>